<commit_message>
Updated Changes in API
</commit_message>
<xml_diff>
--- a/backend/dashboard/Dashboard - Sheet1.xlsx
+++ b/backend/dashboard/Dashboard - Sheet1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Engineering\New folder\Company_details\dashboard\backend\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D0BDC8-CFE6-4D17-AA86-1008352772D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9B06D7-C31C-4645-909A-83CCD13B5870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E4DBBF88-E53C-403A-97C6-DB95538E1A57}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="552">
   <si>
     <t>Initiated</t>
   </si>
@@ -1440,9 +1440,6 @@
   </si>
   <si>
     <t>https://www.amns.in/</t>
-  </si>
-  <si>
-    <t>Tue 10 Feb 2026 2pm – 3pm (IST)</t>
   </si>
   <si>
     <t>called: asked to call next week 18 feb 3pm-3:30 pm: meeting Report:(Less Costing Interest) 
@@ -1455,9 +1452,6 @@
 6. Link(Sent)</t>
   </si>
   <si>
-    <t>10/3/2026 2pm – 3pm</t>
-  </si>
-  <si>
     <t>KBS Certification Services Limited</t>
   </si>
   <si>
@@ -1537,9 +1531,6 @@
     <t>Discuss call</t>
   </si>
   <si>
-    <t>`1</t>
-  </si>
-  <si>
     <t>Specific Services for them required DOC</t>
   </si>
   <si>
@@ -1798,6 +1789,33 @@
   </si>
   <si>
     <t>Meeting Discussion</t>
+  </si>
+  <si>
+    <t>Teleysia Networks Pvt Ltd</t>
+  </si>
+  <si>
+    <t>telecom engineering and consultancy services company</t>
+  </si>
+  <si>
+    <t>https://teleysia.com/</t>
+  </si>
+  <si>
+    <t>chirag@teleysia.com</t>
+  </si>
+  <si>
+    <t>Samit</t>
+  </si>
+  <si>
+    <t>oil and gas geophysical services company</t>
+  </si>
+  <si>
+    <t>http://samit.in</t>
+  </si>
+  <si>
+    <t>Pranaya Sangvai &lt;pranaya.sangvai@samit.in&gt;</t>
+  </si>
+  <si>
+    <t>call on monday 3 march at 10:30 am</t>
   </si>
 </sst>
 </file>
@@ -2670,7 +2688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B8F9747-8500-41E7-983E-FC401CEC534D}">
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="10" max="10" width="9.453125" style="3" bestFit="1" customWidth="1"/>
@@ -2717,7 +2735,7 @@
         <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="O1" t="s">
         <v>13</v>
@@ -2754,9 +2772,6 @@
       <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="3">
-        <v>46086.583333333336</v>
-      </c>
       <c r="K2" t="s">
         <v>24</v>
       </c>
@@ -2767,7 +2782,7 @@
         <v>25</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="P2" t="s">
         <v>26</v>
@@ -2804,9 +2819,6 @@
       <c r="I3" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="3">
-        <v>46085</v>
-      </c>
       <c r="L3" t="s">
         <v>24</v>
       </c>
@@ -2837,7 +2849,7 @@
         <v>35</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="G4" t="s">
         <v>36</v>
@@ -2848,9 +2860,6 @@
       <c r="I4" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>453</v>
-      </c>
       <c r="K4" t="s">
         <v>24</v>
       </c>
@@ -2861,7 +2870,7 @@
         <v>24</v>
       </c>
       <c r="N4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="P4" t="s">
         <v>37</v>
@@ -2895,9 +2904,6 @@
       <c r="I5" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>451</v>
-      </c>
       <c r="K5" t="s">
         <v>24</v>
       </c>
@@ -2908,7 +2914,7 @@
         <v>24</v>
       </c>
       <c r="N5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="P5" t="s">
         <v>37</v>
@@ -2945,9 +2951,6 @@
       <c r="I6" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>477</v>
-      </c>
       <c r="K6" t="s">
         <v>24</v>
       </c>
@@ -2958,10 +2961,10 @@
         <v>24</v>
       </c>
       <c r="N6" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="Q6" t="s">
         <v>49</v>
@@ -3008,7 +3011,7 @@
         <v>95</v>
       </c>
       <c r="P7" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="Q7" t="s">
         <v>24</v>
@@ -3102,7 +3105,7 @@
         <v>67</v>
       </c>
       <c r="P9" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="Q9" t="s">
         <v>24</v>
@@ -3143,13 +3146,13 @@
         <v>24</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="M10" t="s">
         <v>24</v>
       </c>
       <c r="N10" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="P10" t="s">
         <v>72</v>
@@ -3193,7 +3196,7 @@
         <v>24</v>
       </c>
       <c r="N11" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="P11" t="s">
         <v>80</v>
@@ -3237,7 +3240,7 @@
         <v>24</v>
       </c>
       <c r="L12" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="M12" t="s">
         <v>24</v>
@@ -3466,7 +3469,7 @@
         <v>24</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="P17" t="s">
         <v>125</v>
@@ -3492,7 +3495,7 @@
         <v>130</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="L18" s="1" t="s">
         <v>131</v>
@@ -3501,7 +3504,7 @@
         <v>132</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="O18" t="s">
         <v>133</v>
@@ -3592,13 +3595,13 @@
         <v>24</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="M20" t="s">
         <v>24</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="P20" t="s">
         <v>24</v>
@@ -3636,7 +3639,7 @@
         <v>152</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="K21" t="s">
         <v>24</v>
@@ -3683,13 +3686,13 @@
         <v>158</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="M22" t="s">
         <v>24</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="P22" t="s">
         <v>159</v>
@@ -3724,13 +3727,13 @@
         <v>24</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="M23" t="s">
         <v>24</v>
       </c>
       <c r="N23" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="O23" t="s">
         <v>165</v>
@@ -3777,13 +3780,13 @@
         <v>24</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="M24" t="s">
         <v>24</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="P24" t="s">
         <v>173</v>
@@ -3830,7 +3833,7 @@
         <v>24</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="P25" t="s">
         <v>24</v>
@@ -3880,7 +3883,7 @@
         <v>24</v>
       </c>
       <c r="N26" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="P26" t="s">
         <v>24</v>
@@ -3930,7 +3933,7 @@
         <v>24</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="P27" t="s">
         <v>189</v>
@@ -3980,7 +3983,7 @@
         <v>24</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="P28" t="s">
         <v>195</v>
@@ -4397,7 +4400,7 @@
         <v>24</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="P37" t="s">
         <v>24</v>
@@ -4541,7 +4544,7 @@
         <v>24</v>
       </c>
       <c r="N40" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="P40" t="s">
         <v>268</v>
@@ -4667,7 +4670,7 @@
         <v>24</v>
       </c>
       <c r="G43" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="H43" t="s">
         <v>24</v>
@@ -4688,7 +4691,7 @@
         <v>24</v>
       </c>
       <c r="N43" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="P43" t="s">
         <v>24</v>
@@ -4738,7 +4741,7 @@
         <v>24</v>
       </c>
       <c r="N44" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="P44" t="s">
         <v>24</v>
@@ -4788,7 +4791,7 @@
         <v>24</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="P45" t="s">
         <v>24</v>
@@ -4879,13 +4882,13 @@
         <v>312</v>
       </c>
       <c r="L47" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="M47" t="s">
         <v>24</v>
       </c>
       <c r="N47" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="P47" t="s">
         <v>24</v>
@@ -4935,10 +4938,10 @@
         <v>24</v>
       </c>
       <c r="N48" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="P48" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="Q48" t="s">
         <v>24</v>
@@ -4979,7 +4982,7 @@
         <v>24</v>
       </c>
       <c r="L49" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="M49" t="s">
         <v>24</v>
@@ -5196,7 +5199,7 @@
         <v>24</v>
       </c>
       <c r="L54" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="M54" t="s">
         <v>24</v>
@@ -5372,7 +5375,7 @@
         <v>24</v>
       </c>
       <c r="L58" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="M58" t="s">
         <v>24</v>
@@ -5381,7 +5384,7 @@
         <v>368</v>
       </c>
       <c r="P58" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="Q58" t="s">
         <v>24</v>
@@ -5419,7 +5422,7 @@
         <v>24</v>
       </c>
       <c r="L59" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="M59" t="s">
         <v>24</v>
@@ -5469,7 +5472,7 @@
         <v>24</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="M60" t="s">
         <v>24</v>
@@ -5519,7 +5522,7 @@
         <v>24</v>
       </c>
       <c r="L61" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="M61" t="s">
         <v>24</v>
@@ -5569,7 +5572,7 @@
         <v>24</v>
       </c>
       <c r="L62" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="M62" t="s">
         <v>24</v>
@@ -5616,7 +5619,7 @@
         <v>24</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="M63" t="s">
         <v>24</v>
@@ -5660,13 +5663,13 @@
         <v>24</v>
       </c>
       <c r="L64" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="M64" t="s">
         <v>24</v>
       </c>
       <c r="N64" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="P64" t="s">
         <v>24</v>
@@ -5704,7 +5707,7 @@
         <v>402</v>
       </c>
       <c r="N65" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="66" spans="1:16" ht="409.5" x14ac:dyDescent="0.35">
@@ -5733,13 +5736,13 @@
         <v>46084</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="N66" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="P66" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.35">
@@ -5762,10 +5765,10 @@
         <v>413</v>
       </c>
       <c r="N67" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="P67" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.35">
@@ -5823,10 +5826,10 @@
         <v>46071.666666666664</v>
       </c>
       <c r="L69" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="70" spans="1:16" ht="348" x14ac:dyDescent="0.35">
@@ -5852,13 +5855,13 @@
         <v>431</v>
       </c>
       <c r="L70" s="1" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="P70" s="1" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.35">
@@ -5884,7 +5887,7 @@
         <v>437</v>
       </c>
       <c r="P71" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.35">
@@ -5933,27 +5936,27 @@
         <v>46176</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="P73" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
+        <v>452</v>
+      </c>
+      <c r="C74" t="s">
+        <v>453</v>
+      </c>
+      <c r="D74" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="C74" t="s">
+      <c r="E74" t="s">
         <v>455</v>
       </c>
-      <c r="D74" s="4" t="s">
+      <c r="F74" t="s">
         <v>456</v>
-      </c>
-      <c r="E74" t="s">
-        <v>457</v>
-      </c>
-      <c r="F74" t="s">
-        <v>458</v>
       </c>
       <c r="J74" s="3">
         <v>46145</v>
@@ -5961,19 +5964,19 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
+        <v>457</v>
+      </c>
+      <c r="C75" t="s">
+        <v>458</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="E75" t="s">
         <v>459</v>
       </c>
-      <c r="C75" t="s">
+      <c r="F75" t="s">
         <v>460</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>471</v>
-      </c>
-      <c r="E75" t="s">
-        <v>461</v>
-      </c>
-      <c r="F75" t="s">
-        <v>462</v>
       </c>
       <c r="J75" s="3">
         <v>46145</v>
@@ -5981,16 +5984,16 @@
     </row>
     <row r="76" spans="1:16" ht="87" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
+        <v>461</v>
+      </c>
+      <c r="C76" t="s">
+        <v>462</v>
+      </c>
+      <c r="D76" t="s">
+        <v>461</v>
+      </c>
+      <c r="E76" s="1" t="s">
         <v>463</v>
-      </c>
-      <c r="C76" t="s">
-        <v>464</v>
-      </c>
-      <c r="D76" t="s">
-        <v>463</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>465</v>
       </c>
       <c r="J76" s="3">
         <v>46176</v>
@@ -5998,50 +6001,50 @@
     </row>
     <row r="77" spans="1:16" ht="319" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
+        <v>464</v>
+      </c>
+      <c r="C77" t="s">
+        <v>465</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="E77" t="s">
         <v>466</v>
       </c>
-      <c r="C77" t="s">
+      <c r="F77" t="s">
         <v>467</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>470</v>
-      </c>
-      <c r="E77" t="s">
-        <v>468</v>
-      </c>
-      <c r="F77" t="s">
-        <v>469</v>
       </c>
       <c r="J77" s="3">
         <v>46176</v>
       </c>
       <c r="L77" s="1" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="145" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="E78" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="G78" t="s">
         <v>512</v>
-      </c>
-      <c r="G78" t="s">
-        <v>515</v>
       </c>
       <c r="J78" s="3">
         <v>46115</v>
       </c>
       <c r="N78" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="E79" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="J79" s="3">
         <v>46115</v>
@@ -6052,10 +6055,10 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="N80" t="s">
         <v>95</v>
@@ -6063,30 +6066,67 @@
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="L81" t="s">
         <v>221</v>
       </c>
       <c r="N81" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
     </row>
     <row r="82" spans="2:14" ht="188.5" x14ac:dyDescent="0.35">
       <c r="B82" s="1" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="E82" t="s">
+        <v>524</v>
+      </c>
+      <c r="L82" t="s">
         <v>527</v>
       </c>
-      <c r="L82" t="s">
-        <v>530</v>
-      </c>
       <c r="N82" s="1" t="s">
-        <v>529</v>
+        <v>526</v>
+      </c>
+    </row>
+    <row r="83" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B83" t="s">
+        <v>543</v>
+      </c>
+      <c r="C83" t="s">
+        <v>544</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="E83" t="s">
+        <v>546</v>
+      </c>
+      <c r="J83" s="3">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="84" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B84" t="s">
+        <v>547</v>
+      </c>
+      <c r="C84" t="s">
+        <v>548</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="E84" t="s">
+        <v>550</v>
+      </c>
+      <c r="J84" s="3">
+        <v>46084</v>
+      </c>
+      <c r="L84" t="s">
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -6095,6 +6135,8 @@
     <hyperlink ref="D77" r:id="rId2" xr:uid="{F59FD7BD-EF37-422C-B14C-E8B744CC7917}"/>
     <hyperlink ref="D80" r:id="rId3" xr:uid="{06688F0B-3B69-4507-833A-4EBFAD76EA02}"/>
     <hyperlink ref="D81" r:id="rId4" xr:uid="{727AFC24-B8EA-4589-A6F4-171C16112A6A}"/>
+    <hyperlink ref="D83" r:id="rId5" xr:uid="{245D988C-AEF0-4272-B8BC-4730AEB93C50}"/>
+    <hyperlink ref="D84" r:id="rId6" xr:uid="{4E5DCDC6-0DCD-47D9-ACD7-68349C27F8E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>